<commit_message>
Deploy infrastructure-ai-bot with FastAPI and OpenAI integration
</commit_message>
<xml_diff>
--- a/Training_Servers_80Rows.xlsx
+++ b/Training_Servers_80Rows.xlsx
@@ -1,11 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30317"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="1" documentId="11_895317C50A40E800E1B8C888BFD8344068B9AB5E" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4B8D0DA6-8C56-459D-A2C3-16925988D6D0}"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Fajr\Downloads\COOP\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D999670-94C5-44DB-9195-824633B7B297}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="0" windowHeight="0" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="13875" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Training_Data" sheetId="1" r:id="rId1"/>
@@ -1582,11 +1587,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="Arial"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -1627,7 +1632,7 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="عادي" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -1947,12 +1952,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:J81"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="10" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10">
+    <row r="1" spans="1:10" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1984,7 +1989,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:10">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>10</v>
       </c>
@@ -2016,7 +2021,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="3" spans="1:10">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>19</v>
       </c>
@@ -2048,7 +2053,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="4" spans="1:10">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>27</v>
       </c>
@@ -2080,7 +2085,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="5" spans="1:10">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>35</v>
       </c>
@@ -2112,7 +2117,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="6" spans="1:10">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>43</v>
       </c>
@@ -2144,7 +2149,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="7" spans="1:10">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>50</v>
       </c>
@@ -2176,7 +2181,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="8" spans="1:10">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>57</v>
       </c>
@@ -2208,7 +2213,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="9" spans="1:10">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>64</v>
       </c>
@@ -2240,7 +2245,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="10" spans="1:10">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>71</v>
       </c>
@@ -2272,7 +2277,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="11" spans="1:10">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>78</v>
       </c>
@@ -2304,7 +2309,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:10">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>85</v>
       </c>
@@ -2336,7 +2341,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="13" spans="1:10">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>92</v>
       </c>
@@ -2368,7 +2373,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="14" spans="1:10">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>99</v>
       </c>
@@ -2400,7 +2405,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="15" spans="1:10">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>106</v>
       </c>
@@ -2432,7 +2437,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="16" spans="1:10">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>113</v>
       </c>
@@ -2464,7 +2469,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="17" spans="1:10">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>120</v>
       </c>
@@ -2496,7 +2501,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="18" spans="1:10">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>127</v>
       </c>
@@ -2528,7 +2533,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="19" spans="1:10">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>134</v>
       </c>
@@ -2560,7 +2565,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="20" spans="1:10">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>141</v>
       </c>
@@ -2592,7 +2597,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="21" spans="1:10">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>148</v>
       </c>
@@ -2624,7 +2629,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="22" spans="1:10">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>155</v>
       </c>
@@ -2656,7 +2661,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="23" spans="1:10">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>161</v>
       </c>
@@ -2688,7 +2693,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="24" spans="1:10">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>167</v>
       </c>
@@ -2720,7 +2725,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="25" spans="1:10">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>173</v>
       </c>
@@ -2752,7 +2757,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="26" spans="1:10">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>179</v>
       </c>
@@ -2784,7 +2789,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="27" spans="1:10">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>185</v>
       </c>
@@ -2816,7 +2821,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="28" spans="1:10">
+    <row r="28" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>191</v>
       </c>
@@ -2848,7 +2853,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="29" spans="1:10">
+    <row r="29" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>197</v>
       </c>
@@ -2880,7 +2885,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="30" spans="1:10">
+    <row r="30" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>203</v>
       </c>
@@ -2912,7 +2917,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="31" spans="1:10">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>209</v>
       </c>
@@ -2944,7 +2949,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="32" spans="1:10">
+    <row r="32" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>215</v>
       </c>
@@ -2976,7 +2981,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="33" spans="1:10">
+    <row r="33" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>221</v>
       </c>
@@ -3008,7 +3013,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="34" spans="1:10">
+    <row r="34" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>227</v>
       </c>
@@ -3040,7 +3045,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="35" spans="1:10">
+    <row r="35" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>233</v>
       </c>
@@ -3072,7 +3077,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="36" spans="1:10">
+    <row r="36" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>239</v>
       </c>
@@ -3104,7 +3109,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="37" spans="1:10">
+    <row r="37" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>245</v>
       </c>
@@ -3136,7 +3141,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="38" spans="1:10">
+    <row r="38" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>251</v>
       </c>
@@ -3168,7 +3173,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="39" spans="1:10">
+    <row r="39" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>257</v>
       </c>
@@ -3200,7 +3205,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="40" spans="1:10">
+    <row r="40" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>263</v>
       </c>
@@ -3232,7 +3237,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="41" spans="1:10">
+    <row r="41" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>269</v>
       </c>
@@ -3264,7 +3269,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="42" spans="1:10">
+    <row r="42" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>275</v>
       </c>
@@ -3296,7 +3301,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="43" spans="1:10">
+    <row r="43" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>281</v>
       </c>
@@ -3328,7 +3333,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="44" spans="1:10">
+    <row r="44" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>287</v>
       </c>
@@ -3360,7 +3365,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="45" spans="1:10">
+    <row r="45" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>293</v>
       </c>
@@ -3392,7 +3397,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="46" spans="1:10">
+    <row r="46" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>299</v>
       </c>
@@ -3424,7 +3429,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="47" spans="1:10">
+    <row r="47" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>305</v>
       </c>
@@ -3456,7 +3461,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="48" spans="1:10">
+    <row r="48" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>311</v>
       </c>
@@ -3488,7 +3493,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="49" spans="1:10">
+    <row r="49" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>317</v>
       </c>
@@ -3520,7 +3525,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="50" spans="1:10">
+    <row r="50" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
         <v>323</v>
       </c>
@@ -3552,7 +3557,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="51" spans="1:10">
+    <row r="51" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>329</v>
       </c>
@@ -3584,7 +3589,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="52" spans="1:10">
+    <row r="52" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
         <v>335</v>
       </c>
@@ -3616,7 +3621,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="53" spans="1:10">
+    <row r="53" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
         <v>341</v>
       </c>
@@ -3648,7 +3653,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="54" spans="1:10">
+    <row r="54" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
         <v>347</v>
       </c>
@@ -3680,7 +3685,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="55" spans="1:10">
+    <row r="55" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
         <v>353</v>
       </c>
@@ -3712,7 +3717,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="56" spans="1:10">
+    <row r="56" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
         <v>359</v>
       </c>
@@ -3744,7 +3749,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="57" spans="1:10">
+    <row r="57" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
         <v>365</v>
       </c>
@@ -3776,7 +3781,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="58" spans="1:10">
+    <row r="58" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
         <v>371</v>
       </c>
@@ -3808,7 +3813,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="59" spans="1:10">
+    <row r="59" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
         <v>377</v>
       </c>
@@ -3840,7 +3845,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="60" spans="1:10">
+    <row r="60" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
         <v>383</v>
       </c>
@@ -3872,7 +3877,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="61" spans="1:10">
+    <row r="61" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
         <v>389</v>
       </c>
@@ -3904,7 +3909,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="62" spans="1:10">
+    <row r="62" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
         <v>395</v>
       </c>
@@ -3936,7 +3941,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="63" spans="1:10">
+    <row r="63" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
         <v>401</v>
       </c>
@@ -3968,7 +3973,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="64" spans="1:10">
+    <row r="64" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
         <v>407</v>
       </c>
@@ -4000,7 +4005,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="65" spans="1:10">
+    <row r="65" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
         <v>413</v>
       </c>
@@ -4032,7 +4037,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="66" spans="1:10">
+    <row r="66" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
         <v>419</v>
       </c>
@@ -4064,7 +4069,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="67" spans="1:10">
+    <row r="67" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
         <v>425</v>
       </c>
@@ -4096,7 +4101,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="68" spans="1:10">
+    <row r="68" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
         <v>431</v>
       </c>
@@ -4128,7 +4133,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="69" spans="1:10">
+    <row r="69" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
         <v>437</v>
       </c>
@@ -4160,7 +4165,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="70" spans="1:10">
+    <row r="70" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
         <v>443</v>
       </c>
@@ -4192,7 +4197,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="71" spans="1:10">
+    <row r="71" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
         <v>449</v>
       </c>
@@ -4224,7 +4229,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="72" spans="1:10">
+    <row r="72" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
         <v>455</v>
       </c>
@@ -4256,7 +4261,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="73" spans="1:10">
+    <row r="73" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
         <v>461</v>
       </c>
@@ -4288,7 +4293,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="74" spans="1:10">
+    <row r="74" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
         <v>467</v>
       </c>
@@ -4320,7 +4325,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="75" spans="1:10">
+    <row r="75" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
         <v>473</v>
       </c>
@@ -4352,7 +4357,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="76" spans="1:10">
+    <row r="76" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
         <v>479</v>
       </c>
@@ -4384,7 +4389,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="77" spans="1:10">
+    <row r="77" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
         <v>485</v>
       </c>
@@ -4416,7 +4421,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="78" spans="1:10">
+    <row r="78" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A78" t="s">
         <v>491</v>
       </c>
@@ -4448,7 +4453,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="79" spans="1:10">
+    <row r="79" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A79" t="s">
         <v>497</v>
       </c>
@@ -4480,7 +4485,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="80" spans="1:10">
+    <row r="80" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A80" t="s">
         <v>503</v>
       </c>
@@ -4512,7 +4517,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="81" spans="1:10">
+    <row r="81" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A81" t="s">
         <v>509</v>
       </c>

</xml_diff>